<commit_message>
Update Plan Entrega IS y TD 2026.xlsx
</commit_message>
<xml_diff>
--- a/Documentación/Plan Entrega IS y TD 2026.xlsx
+++ b/Documentación/Plan Entrega IS y TD 2026.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30105"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{120A94D2-8947-42D8-8C4F-2DF98F743A79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26FEBDBA-A43F-44AD-9D25-AFFE45AA8F7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" tabRatio="699" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" tabRatio="699" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan Entregas IS 2026" sheetId="2" r:id="rId1"/>
     <sheet name="Plan de entregas TD 2026" sheetId="7" r:id="rId2"/>
+    <sheet name="Cronograma" sheetId="8" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -32,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="117">
   <si>
     <t>Iteración</t>
   </si>
@@ -362,12 +363,48 @@
   <si>
     <t>Planificación TD  - 2026</t>
   </si>
+  <si>
+    <t>Clase</t>
+  </si>
+  <si>
+    <t>Fecha</t>
+  </si>
+  <si>
+    <t>Tema</t>
+  </si>
+  <si>
+    <t>Introducción</t>
+  </si>
+  <si>
+    <t>Recuperatorio</t>
+  </si>
+  <si>
+    <t>Entrega 1</t>
+  </si>
+  <si>
+    <t>Parcial 1</t>
+  </si>
+  <si>
+    <t>Entrega 2</t>
+  </si>
+  <si>
+    <t>Parcial 2</t>
+  </si>
+  <si>
+    <t>Entrega 3</t>
+  </si>
+  <si>
+    <t>FERIADO</t>
+  </si>
+  <si>
+    <t>Implementacion.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -383,8 +420,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -403,6 +447,24 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="37">
     <border>
@@ -872,7 +934,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="74">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -974,6 +1036,13 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="36" xfId="0" applyBorder="1"/>
+    <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="16" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="16" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="16" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1033,6 +1102,22 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1347,13 +1432,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="48" t="s">
         <v>100</v>
       </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
     </row>
     <row r="2" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -1373,61 +1458,61 @@
       </c>
     </row>
     <row r="3" spans="1:5" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="51">
+      <c r="A3" s="68">
         <v>1</v>
       </c>
-      <c r="B3" s="19"/>
-      <c r="C3" s="18" t="s">
+      <c r="B3" s="69"/>
+      <c r="C3" s="70" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="21" t="s">
+      <c r="D3" s="71" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="18" t="s">
+      <c r="E3" s="70" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="51"/>
-      <c r="B4" s="19"/>
-      <c r="C4" s="18" t="s">
+      <c r="A4" s="68"/>
+      <c r="B4" s="69"/>
+      <c r="C4" s="70" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="21" t="s">
+      <c r="D4" s="71" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="18" t="s">
+      <c r="E4" s="70" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="51"/>
-      <c r="B5" s="19"/>
-      <c r="C5" s="3" t="s">
+      <c r="A5" s="68"/>
+      <c r="B5" s="69"/>
+      <c r="C5" s="72" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="D5" s="73" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="18" t="s">
+      <c r="E5" s="70" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="51"/>
-      <c r="B6" s="19"/>
-      <c r="C6" s="18" t="s">
+      <c r="A6" s="68"/>
+      <c r="B6" s="69"/>
+      <c r="C6" s="70" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="21" t="s">
+      <c r="D6" s="71" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="18" t="s">
+      <c r="E6" s="70" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="56">
+      <c r="A7" s="63">
         <v>2</v>
       </c>
       <c r="B7" s="19"/>
@@ -1442,7 +1527,7 @@
       </c>
     </row>
     <row r="8" spans="1:5" ht="270.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="57"/>
+      <c r="A8" s="64"/>
       <c r="B8" s="19"/>
       <c r="C8" s="4" t="s">
         <v>19</v>
@@ -1455,7 +1540,7 @@
       </c>
     </row>
     <row r="9" spans="1:5" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="57"/>
+      <c r="A9" s="64"/>
       <c r="B9" s="19"/>
       <c r="C9" s="18" t="s">
         <v>21</v>
@@ -1468,7 +1553,7 @@
       </c>
     </row>
     <row r="10" spans="1:5" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="57"/>
+      <c r="A10" s="64"/>
       <c r="B10" s="19"/>
       <c r="C10" s="18" t="s">
         <v>24</v>
@@ -1476,10 +1561,12 @@
       <c r="D10" s="21" t="s">
         <v>101</v>
       </c>
-      <c r="E10" s="18"/>
+      <c r="E10" s="18" t="s">
+        <v>116</v>
+      </c>
     </row>
     <row r="11" spans="1:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="58"/>
+      <c r="A11" s="65"/>
       <c r="B11" s="19"/>
       <c r="C11" s="18" t="s">
         <v>25</v>
@@ -1492,7 +1579,7 @@
       </c>
     </row>
     <row r="12" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="52">
+      <c r="A12" s="59">
         <v>3</v>
       </c>
       <c r="B12" s="19"/>
@@ -1507,7 +1594,7 @@
       </c>
     </row>
     <row r="13" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="51"/>
+      <c r="A13" s="58"/>
       <c r="B13" s="19"/>
       <c r="C13" s="4" t="s">
         <v>29</v>
@@ -1520,7 +1607,7 @@
       </c>
     </row>
     <row r="14" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="51"/>
+      <c r="A14" s="58"/>
       <c r="B14" s="19"/>
       <c r="C14" s="18" t="s">
         <v>25</v>
@@ -1533,7 +1620,7 @@
       </c>
     </row>
     <row r="15" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="51"/>
+      <c r="A15" s="58"/>
       <c r="B15" s="19"/>
       <c r="C15" s="18" t="s">
         <v>30</v>
@@ -1546,7 +1633,7 @@
       </c>
     </row>
     <row r="16" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="53"/>
+      <c r="A16" s="60"/>
       <c r="B16" s="19"/>
       <c r="C16" s="18" t="s">
         <v>33</v>
@@ -1559,21 +1646,21 @@
       </c>
     </row>
     <row r="17" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="47" t="s">
+      <c r="A17" s="54" t="s">
         <v>36</v>
       </c>
-      <c r="B17" s="47"/>
-      <c r="C17" s="47"/>
-      <c r="D17" s="47"/>
+      <c r="B17" s="54"/>
+      <c r="C17" s="54"/>
+      <c r="D17" s="54"/>
     </row>
     <row r="18" spans="1:4" ht="45" x14ac:dyDescent="0.25">
       <c r="A18" s="9">
         <v>1</v>
       </c>
-      <c r="B18" s="48" t="s">
+      <c r="B18" s="55" t="s">
         <v>37</v>
       </c>
-      <c r="C18" s="49"/>
+      <c r="C18" s="56"/>
       <c r="D18" s="5" t="s">
         <v>38</v>
       </c>
@@ -1582,10 +1669,10 @@
       <c r="A19" s="10">
         <v>2</v>
       </c>
-      <c r="B19" s="54" t="s">
+      <c r="B19" s="61" t="s">
         <v>39</v>
       </c>
-      <c r="C19" s="55"/>
+      <c r="C19" s="62"/>
       <c r="D19" s="6" t="s">
         <v>40</v>
       </c>
@@ -1594,10 +1681,10 @@
       <c r="A20" s="11">
         <v>3</v>
       </c>
-      <c r="B20" s="44" t="s">
+      <c r="B20" s="51" t="s">
         <v>41</v>
       </c>
-      <c r="C20" s="50"/>
+      <c r="C20" s="57"/>
       <c r="D20" s="7" t="s">
         <v>42</v>
       </c>
@@ -1606,10 +1693,10 @@
       <c r="A21" s="11">
         <v>4</v>
       </c>
-      <c r="B21" s="43" t="s">
+      <c r="B21" s="50" t="s">
         <v>43</v>
       </c>
-      <c r="C21" s="44"/>
+      <c r="C21" s="51"/>
       <c r="D21" s="7" t="s">
         <v>44</v>
       </c>
@@ -1618,10 +1705,10 @@
       <c r="A22" s="11">
         <v>5</v>
       </c>
-      <c r="B22" s="43" t="s">
+      <c r="B22" s="50" t="s">
         <v>45</v>
       </c>
-      <c r="C22" s="44"/>
+      <c r="C22" s="51"/>
       <c r="D22" s="7" t="s">
         <v>46</v>
       </c>
@@ -1630,10 +1717,10 @@
       <c r="A23" s="11">
         <v>6</v>
       </c>
-      <c r="B23" s="43" t="s">
+      <c r="B23" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="C23" s="44"/>
+      <c r="C23" s="51"/>
       <c r="D23" s="7" t="s">
         <v>48</v>
       </c>
@@ -1654,10 +1741,10 @@
       <c r="A25" s="11">
         <v>7</v>
       </c>
-      <c r="B25" s="43" t="s">
+      <c r="B25" s="50" t="s">
         <v>51</v>
       </c>
-      <c r="C25" s="44"/>
+      <c r="C25" s="51"/>
       <c r="D25" s="7" t="s">
         <v>52</v>
       </c>
@@ -1666,10 +1753,10 @@
       <c r="A26" s="11">
         <v>8</v>
       </c>
-      <c r="B26" s="43" t="s">
+      <c r="B26" s="50" t="s">
         <v>53</v>
       </c>
-      <c r="C26" s="44"/>
+      <c r="C26" s="51"/>
       <c r="D26" s="7" t="s">
         <v>54</v>
       </c>
@@ -1678,10 +1765,10 @@
       <c r="A27" s="12">
         <v>9</v>
       </c>
-      <c r="B27" s="45" t="s">
+      <c r="B27" s="52" t="s">
         <v>55</v>
       </c>
-      <c r="C27" s="46"/>
+      <c r="C27" s="53"/>
       <c r="D27" s="8" t="s">
         <v>56</v>
       </c>
@@ -1720,13 +1807,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="41" t="s">
+      <c r="A1" s="48" t="s">
         <v>104</v>
       </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
+      <c r="D1" s="49"/>
+      <c r="E1" s="49"/>
     </row>
     <row r="2" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="15" t="s">
@@ -1761,7 +1848,7 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="56">
+      <c r="A4" s="63">
         <v>1</v>
       </c>
       <c r="B4" s="31"/>
@@ -1776,7 +1863,7 @@
       </c>
     </row>
     <row r="5" spans="1:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="57"/>
+      <c r="A5" s="64"/>
       <c r="B5" s="31"/>
       <c r="C5" s="18" t="s">
         <v>63</v>
@@ -1789,7 +1876,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="57"/>
+      <c r="A6" s="64"/>
       <c r="B6" s="40"/>
       <c r="C6" s="18" t="s">
         <v>65</v>
@@ -1800,7 +1887,7 @@
       <c r="E6" s="18"/>
     </row>
     <row r="7" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="57"/>
+      <c r="A7" s="64"/>
       <c r="B7" s="32"/>
       <c r="C7" s="18" t="s">
         <v>67</v>
@@ -1811,7 +1898,7 @@
       <c r="E7" s="21"/>
     </row>
     <row r="8" spans="1:5" ht="180.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="57"/>
+      <c r="A8" s="64"/>
       <c r="B8" s="33"/>
       <c r="C8" s="24" t="s">
         <v>69</v>
@@ -1822,7 +1909,7 @@
       <c r="E8" s="25"/>
     </row>
     <row r="9" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="57"/>
+      <c r="A9" s="64"/>
       <c r="B9" s="34"/>
       <c r="C9" s="18" t="s">
         <v>71</v>
@@ -1833,7 +1920,7 @@
       <c r="E9" s="21"/>
     </row>
     <row r="10" spans="1:5" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="58"/>
+      <c r="A10" s="65"/>
       <c r="B10" s="31"/>
       <c r="C10" s="30" t="s">
         <v>73</v>
@@ -1846,7 +1933,7 @@
       </c>
     </row>
     <row r="11" spans="1:5" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="52">
+      <c r="A11" s="59">
         <v>2</v>
       </c>
       <c r="B11" s="19"/>
@@ -1861,7 +1948,7 @@
       </c>
     </row>
     <row r="12" spans="1:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="53"/>
+      <c r="A12" s="60"/>
       <c r="B12" s="19"/>
       <c r="C12" s="18" t="s">
         <v>77</v>
@@ -1874,7 +1961,7 @@
       </c>
     </row>
     <row r="13" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="52">
+      <c r="A13" s="59">
         <v>3</v>
       </c>
       <c r="B13" s="35"/>
@@ -1889,7 +1976,7 @@
       </c>
     </row>
     <row r="14" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="51"/>
+      <c r="A14" s="58"/>
       <c r="B14" s="36"/>
       <c r="C14" s="28" t="s">
         <v>83</v>
@@ -1902,7 +1989,7 @@
       </c>
     </row>
     <row r="15" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="51"/>
+      <c r="A15" s="58"/>
       <c r="B15" s="37"/>
       <c r="C15" s="26" t="s">
         <v>86</v>
@@ -1915,7 +2002,7 @@
       </c>
     </row>
     <row r="16" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="51"/>
+      <c r="A16" s="58"/>
       <c r="B16" s="37"/>
       <c r="C16" s="26" t="s">
         <v>88</v>
@@ -1928,7 +2015,7 @@
       </c>
     </row>
     <row r="17" spans="1:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="51"/>
+      <c r="A17" s="58"/>
       <c r="B17" s="37"/>
       <c r="C17" s="29" t="s">
         <v>77</v>
@@ -1941,7 +2028,7 @@
       </c>
     </row>
     <row r="18" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="51"/>
+      <c r="A18" s="58"/>
       <c r="B18" s="37"/>
       <c r="C18" s="26" t="s">
         <v>90</v>
@@ -1954,7 +2041,7 @@
       </c>
     </row>
     <row r="19" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="51"/>
+      <c r="A19" s="58"/>
       <c r="B19" s="37"/>
       <c r="C19" s="26" t="s">
         <v>92</v>
@@ -1965,7 +2052,7 @@
       <c r="E19" s="18"/>
     </row>
     <row r="20" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="51"/>
+      <c r="A20" s="58"/>
       <c r="B20" s="37"/>
       <c r="C20" s="18" t="s">
         <v>94</v>
@@ -1978,7 +2065,7 @@
       </c>
     </row>
     <row r="21" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="51"/>
+      <c r="A21" s="58"/>
       <c r="B21" s="38"/>
       <c r="C21" s="18" t="s">
         <v>96</v>
@@ -1991,21 +2078,21 @@
       </c>
     </row>
     <row r="22" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="47" t="s">
+      <c r="A22" s="54" t="s">
         <v>98</v>
       </c>
-      <c r="B22" s="47"/>
-      <c r="C22" s="47"/>
-      <c r="D22" s="47"/>
+      <c r="B22" s="54"/>
+      <c r="C22" s="54"/>
+      <c r="D22" s="54"/>
     </row>
     <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="9">
         <v>1</v>
       </c>
-      <c r="B23" s="59" t="s">
+      <c r="B23" s="66" t="s">
         <v>39</v>
       </c>
-      <c r="C23" s="60"/>
+      <c r="C23" s="67"/>
       <c r="D23" s="5" t="s">
         <v>40</v>
       </c>
@@ -2014,10 +2101,10 @@
       <c r="A24" s="11">
         <v>2</v>
       </c>
-      <c r="B24" s="43" t="s">
+      <c r="B24" s="50" t="s">
         <v>41</v>
       </c>
-      <c r="C24" s="44"/>
+      <c r="C24" s="51"/>
       <c r="D24" s="7" t="s">
         <v>42</v>
       </c>
@@ -2026,10 +2113,10 @@
       <c r="A25" s="11">
         <v>3</v>
       </c>
-      <c r="B25" s="43" t="s">
+      <c r="B25" s="50" t="s">
         <v>43</v>
       </c>
-      <c r="C25" s="44"/>
+      <c r="C25" s="51"/>
       <c r="D25" s="7" t="s">
         <v>44</v>
       </c>
@@ -2038,10 +2125,10 @@
       <c r="A26" s="11">
         <v>4</v>
       </c>
-      <c r="B26" s="43" t="s">
+      <c r="B26" s="50" t="s">
         <v>45</v>
       </c>
-      <c r="C26" s="44"/>
+      <c r="C26" s="51"/>
       <c r="D26" s="7" t="s">
         <v>46</v>
       </c>
@@ -2050,10 +2137,10 @@
       <c r="A27" s="11">
         <v>5</v>
       </c>
-      <c r="B27" s="43" t="s">
+      <c r="B27" s="50" t="s">
         <v>47</v>
       </c>
-      <c r="C27" s="44"/>
+      <c r="C27" s="51"/>
       <c r="D27" s="7" t="s">
         <v>48</v>
       </c>
@@ -2062,10 +2149,10 @@
       <c r="A28" s="11">
         <v>6</v>
       </c>
-      <c r="B28" s="43" t="s">
+      <c r="B28" s="50" t="s">
         <v>51</v>
       </c>
-      <c r="C28" s="44"/>
+      <c r="C28" s="51"/>
       <c r="D28" s="7" t="s">
         <v>52</v>
       </c>
@@ -2074,10 +2161,10 @@
       <c r="A29" s="11">
         <v>7</v>
       </c>
-      <c r="B29" s="43" t="s">
+      <c r="B29" s="50" t="s">
         <v>53</v>
       </c>
-      <c r="C29" s="44"/>
+      <c r="C29" s="51"/>
       <c r="D29" s="7" t="s">
         <v>54</v>
       </c>
@@ -2086,10 +2173,10 @@
       <c r="A30" s="12">
         <v>8</v>
       </c>
-      <c r="B30" s="45" t="s">
+      <c r="B30" s="52" t="s">
         <v>55</v>
       </c>
-      <c r="C30" s="46"/>
+      <c r="C30" s="53"/>
       <c r="D30" s="8" t="s">
         <v>99</v>
       </c>
@@ -2113,4 +2200,172 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F854E2D-0B73-46F0-A47C-EC8E21F4946D}">
+  <dimension ref="A1:C16"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="13.5703125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C1" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" s="41">
+        <v>46121</v>
+      </c>
+      <c r="C2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="41">
+        <v>46128</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" s="41">
+        <v>46135</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="46">
+        <v>4</v>
+      </c>
+      <c r="B5" s="47">
+        <v>46142</v>
+      </c>
+      <c r="C5" s="46" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" s="41">
+        <v>46149</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" s="41">
+        <v>46156</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="44">
+        <v>7</v>
+      </c>
+      <c r="B8" s="45">
+        <v>46163</v>
+      </c>
+      <c r="C8" s="44" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" s="41">
+        <v>46170</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" s="41">
+        <v>46177</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="46">
+        <v>10</v>
+      </c>
+      <c r="B11" s="47">
+        <v>46184</v>
+      </c>
+      <c r="C11" s="46" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" s="41">
+        <v>46191</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="44">
+        <v>12</v>
+      </c>
+      <c r="B13" s="45">
+        <v>46198</v>
+      </c>
+      <c r="C13" s="44" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="46">
+        <v>13</v>
+      </c>
+      <c r="B14" s="47">
+        <v>46205</v>
+      </c>
+      <c r="C14" s="46" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="42">
+        <v>14</v>
+      </c>
+      <c r="B15" s="43">
+        <v>46212</v>
+      </c>
+      <c r="C15" s="42" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="44">
+        <v>15</v>
+      </c>
+      <c r="B16" s="45">
+        <v>46219</v>
+      </c>
+      <c r="C16" s="44" t="s">
+        <v>109</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Carga de frm ControlCambios y BackUp-Restore
</commit_message>
<xml_diff>
--- a/Documentación/Plan Entrega IS y TD 2026.xlsx
+++ b/Documentación/Plan Entrega IS y TD 2026.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30105"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30026"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26FEBDBA-A43F-44AD-9D25-AFFE45AA8F7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" tabRatio="699" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="699" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan Entregas IS 2026" sheetId="2" r:id="rId1"/>
@@ -1043,69 +1043,6 @@
     <xf numFmtId="16" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="16" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1118,6 +1055,69 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="9" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1424,23 +1424,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E27"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="64.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="103.7109375" customWidth="1"/>
-    <col min="5" max="5" width="66.28515625" style="17" customWidth="1"/>
+    <col min="3" max="3" width="64.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="103.6640625" customWidth="1"/>
+    <col min="5" max="5" width="66.33203125" style="17" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+    <row r="1" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="53" t="s">
         <v>100</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-    </row>
-    <row r="2" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="54"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="54"/>
+      <c r="E1" s="54"/>
+    </row>
+    <row r="2" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1457,62 +1457,62 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="68">
+    <row r="3" spans="1:5" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="63">
         <v>1</v>
       </c>
-      <c r="B3" s="69"/>
-      <c r="C3" s="70" t="s">
+      <c r="B3" s="48"/>
+      <c r="C3" s="49" t="s">
         <v>5</v>
       </c>
-      <c r="D3" s="71" t="s">
+      <c r="D3" s="50" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="70" t="s">
+      <c r="E3" s="49" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="68"/>
-      <c r="B4" s="69"/>
-      <c r="C4" s="70" t="s">
+    <row r="4" spans="1:5" ht="101.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="63"/>
+      <c r="B4" s="48"/>
+      <c r="C4" s="49" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="71" t="s">
+      <c r="D4" s="50" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="70" t="s">
+      <c r="E4" s="49" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="68"/>
-      <c r="B5" s="69"/>
-      <c r="C5" s="72" t="s">
+    <row r="5" spans="1:5" ht="87" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="63"/>
+      <c r="B5" s="48"/>
+      <c r="C5" s="51" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="73" t="s">
+      <c r="D5" s="52" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="70" t="s">
+      <c r="E5" s="49" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="105.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="68"/>
-      <c r="B6" s="69"/>
-      <c r="C6" s="70" t="s">
+    <row r="6" spans="1:5" ht="87" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="63"/>
+      <c r="B6" s="48"/>
+      <c r="C6" s="49" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="71" t="s">
+      <c r="D6" s="50" t="s">
         <v>15</v>
       </c>
-      <c r="E6" s="70" t="s">
+      <c r="E6" s="49" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="63">
+    <row r="7" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="69">
         <v>2</v>
       </c>
       <c r="B7" s="19"/>
@@ -1526,8 +1526,8 @@
         <v>13</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="270.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="64"/>
+    <row r="8" spans="1:5" ht="231" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="70"/>
       <c r="B8" s="19"/>
       <c r="C8" s="4" t="s">
         <v>19</v>
@@ -1539,8 +1539,8 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="64"/>
+    <row r="9" spans="1:5" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="70"/>
       <c r="B9" s="19"/>
       <c r="C9" s="18" t="s">
         <v>21</v>
@@ -1552,8 +1552,8 @@
         <v>23</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="75.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="64"/>
+    <row r="10" spans="1:5" ht="58.2" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="70"/>
       <c r="B10" s="19"/>
       <c r="C10" s="18" t="s">
         <v>24</v>
@@ -1565,8 +1565,8 @@
         <v>116</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="65"/>
+    <row r="11" spans="1:5" ht="87" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="71"/>
       <c r="B11" s="19"/>
       <c r="C11" s="18" t="s">
         <v>25</v>
@@ -1578,8 +1578,8 @@
         <v>27</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="59">
+    <row r="12" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="64">
         <v>3</v>
       </c>
       <c r="B12" s="19"/>
@@ -1593,8 +1593,8 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="58"/>
+    <row r="13" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="65"/>
       <c r="B13" s="19"/>
       <c r="C13" s="4" t="s">
         <v>29</v>
@@ -1606,8 +1606,8 @@
         <v>13</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="58"/>
+    <row r="14" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="65"/>
       <c r="B14" s="19"/>
       <c r="C14" s="18" t="s">
         <v>25</v>
@@ -1619,8 +1619,8 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="58"/>
+    <row r="15" spans="1:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="65"/>
       <c r="B15" s="19"/>
       <c r="C15" s="18" t="s">
         <v>30</v>
@@ -1632,8 +1632,8 @@
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="60"/>
+    <row r="16" spans="1:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="66"/>
       <c r="B16" s="19"/>
       <c r="C16" s="18" t="s">
         <v>33</v>
@@ -1645,87 +1645,87 @@
         <v>35</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="54" t="s">
+    <row r="17" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="59" t="s">
         <v>36</v>
       </c>
-      <c r="B17" s="54"/>
-      <c r="C17" s="54"/>
-      <c r="D17" s="54"/>
-    </row>
-    <row r="18" spans="1:4" ht="45" x14ac:dyDescent="0.25">
+      <c r="B17" s="59"/>
+      <c r="C17" s="59"/>
+      <c r="D17" s="59"/>
+    </row>
+    <row r="18" spans="1:4" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A18" s="9">
         <v>1</v>
       </c>
-      <c r="B18" s="55" t="s">
+      <c r="B18" s="60" t="s">
         <v>37</v>
       </c>
-      <c r="C18" s="56"/>
+      <c r="C18" s="61"/>
       <c r="D18" s="5" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="10">
         <v>2</v>
       </c>
-      <c r="B19" s="61" t="s">
+      <c r="B19" s="67" t="s">
         <v>39</v>
       </c>
-      <c r="C19" s="62"/>
+      <c r="C19" s="68"/>
       <c r="D19" s="6" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="11">
         <v>3</v>
       </c>
-      <c r="B20" s="51" t="s">
+      <c r="B20" s="56" t="s">
         <v>41</v>
       </c>
-      <c r="C20" s="57"/>
+      <c r="C20" s="62"/>
       <c r="D20" s="7" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="11">
         <v>4</v>
       </c>
-      <c r="B21" s="50" t="s">
+      <c r="B21" s="55" t="s">
         <v>43</v>
       </c>
-      <c r="C21" s="51"/>
+      <c r="C21" s="56"/>
       <c r="D21" s="7" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="11">
         <v>5</v>
       </c>
-      <c r="B22" s="50" t="s">
+      <c r="B22" s="55" t="s">
         <v>45</v>
       </c>
-      <c r="C22" s="51"/>
+      <c r="C22" s="56"/>
       <c r="D22" s="7" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="11">
         <v>6</v>
       </c>
-      <c r="B23" s="50" t="s">
+      <c r="B23" s="55" t="s">
         <v>47</v>
       </c>
-      <c r="C23" s="51"/>
+      <c r="C23" s="56"/>
       <c r="D23" s="7" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="11">
         <v>6</v>
       </c>
@@ -1737,38 +1737,38 @@
         <v>50</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="11">
         <v>7</v>
       </c>
-      <c r="B25" s="50" t="s">
+      <c r="B25" s="55" t="s">
         <v>51</v>
       </c>
-      <c r="C25" s="51"/>
+      <c r="C25" s="56"/>
       <c r="D25" s="7" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A26" s="11">
         <v>8</v>
       </c>
-      <c r="B26" s="50" t="s">
+      <c r="B26" s="55" t="s">
         <v>53</v>
       </c>
-      <c r="C26" s="51"/>
+      <c r="C26" s="56"/>
       <c r="D26" s="7" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A27" s="12">
         <v>9</v>
       </c>
-      <c r="B27" s="52" t="s">
+      <c r="B27" s="57" t="s">
         <v>55</v>
       </c>
-      <c r="C27" s="53"/>
+      <c r="C27" s="58"/>
       <c r="D27" s="8" t="s">
         <v>56</v>
       </c>
@@ -1798,24 +1798,24 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07CA6276-71FC-4BB7-B5A8-70E7B7E3AFEC}">
   <dimension ref="A1:E30"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11.5703125" style="16"/>
-    <col min="3" max="3" width="67.42578125" customWidth="1"/>
-    <col min="4" max="4" width="96.28515625" style="14" customWidth="1"/>
-    <col min="5" max="5" width="62.85546875" customWidth="1"/>
+    <col min="1" max="1" width="11.5546875" style="16"/>
+    <col min="3" max="3" width="67.44140625" customWidth="1"/>
+    <col min="4" max="4" width="96.33203125" style="14" customWidth="1"/>
+    <col min="5" max="5" width="62.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="48" t="s">
+    <row r="1" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="53" t="s">
         <v>104</v>
       </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
-      <c r="E1" s="49"/>
-    </row>
-    <row r="2" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="54"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="54"/>
+      <c r="E1" s="54"/>
+    </row>
+    <row r="2" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="15" t="s">
         <v>57</v>
       </c>
@@ -1832,7 +1832,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3" s="39">
         <v>0</v>
       </c>
@@ -1847,8 +1847,8 @@
         <v>60</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="63">
+    <row r="4" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="69">
         <v>1</v>
       </c>
       <c r="B4" s="31"/>
@@ -1862,8 +1862,8 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="64"/>
+    <row r="5" spans="1:5" ht="87" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="70"/>
       <c r="B5" s="31"/>
       <c r="C5" s="18" t="s">
         <v>63</v>
@@ -1875,8 +1875,8 @@
         <v>60</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="64"/>
+    <row r="6" spans="1:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="70"/>
       <c r="B6" s="40"/>
       <c r="C6" s="18" t="s">
         <v>65</v>
@@ -1886,8 +1886,8 @@
       </c>
       <c r="E6" s="18"/>
     </row>
-    <row r="7" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="64"/>
+    <row r="7" spans="1:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="70"/>
       <c r="B7" s="32"/>
       <c r="C7" s="18" t="s">
         <v>67</v>
@@ -1897,8 +1897,8 @@
       </c>
       <c r="E7" s="21"/>
     </row>
-    <row r="8" spans="1:5" ht="180.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="64"/>
+    <row r="8" spans="1:5" ht="130.19999999999999" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="70"/>
       <c r="B8" s="33"/>
       <c r="C8" s="24" t="s">
         <v>69</v>
@@ -1908,8 +1908,8 @@
       </c>
       <c r="E8" s="25"/>
     </row>
-    <row r="9" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="64"/>
+    <row r="9" spans="1:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="70"/>
       <c r="B9" s="34"/>
       <c r="C9" s="18" t="s">
         <v>71</v>
@@ -1919,8 +1919,8 @@
       </c>
       <c r="E9" s="21"/>
     </row>
-    <row r="10" spans="1:5" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="65"/>
+    <row r="10" spans="1:5" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A10" s="71"/>
       <c r="B10" s="31"/>
       <c r="C10" s="30" t="s">
         <v>73</v>
@@ -1932,8 +1932,8 @@
         <v>75</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="59">
+    <row r="11" spans="1:5" ht="43.8" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A11" s="64">
         <v>2</v>
       </c>
       <c r="B11" s="19"/>
@@ -1947,8 +1947,8 @@
         <v>103</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="60"/>
+    <row r="12" spans="1:5" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A12" s="66"/>
       <c r="B12" s="19"/>
       <c r="C12" s="18" t="s">
         <v>77</v>
@@ -1960,8 +1960,8 @@
         <v>79</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="59">
+    <row r="13" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A13" s="64">
         <v>3</v>
       </c>
       <c r="B13" s="35"/>
@@ -1975,8 +1975,8 @@
         <v>82</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="58"/>
+    <row r="14" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="65"/>
       <c r="B14" s="36"/>
       <c r="C14" s="28" t="s">
         <v>83</v>
@@ -1988,8 +1988,8 @@
         <v>85</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="58"/>
+    <row r="15" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="65"/>
       <c r="B15" s="37"/>
       <c r="C15" s="26" t="s">
         <v>86</v>
@@ -2001,8 +2001,8 @@
         <v>85</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="58"/>
+    <row r="16" spans="1:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="65"/>
       <c r="B16" s="37"/>
       <c r="C16" s="26" t="s">
         <v>88</v>
@@ -2014,8 +2014,8 @@
         <v>85</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="58"/>
+    <row r="17" spans="1:5" ht="72.599999999999994" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="65"/>
       <c r="B17" s="37"/>
       <c r="C17" s="29" t="s">
         <v>77</v>
@@ -2027,8 +2027,8 @@
         <v>85</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="58"/>
+    <row r="18" spans="1:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="65"/>
       <c r="B18" s="37"/>
       <c r="C18" s="26" t="s">
         <v>90</v>
@@ -2040,8 +2040,8 @@
         <v>85</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="58"/>
+    <row r="19" spans="1:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="65"/>
       <c r="B19" s="37"/>
       <c r="C19" s="26" t="s">
         <v>92</v>
@@ -2051,8 +2051,8 @@
       </c>
       <c r="E19" s="18"/>
     </row>
-    <row r="20" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="58"/>
+    <row r="20" spans="1:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="65"/>
       <c r="B20" s="37"/>
       <c r="C20" s="18" t="s">
         <v>94</v>
@@ -2064,8 +2064,8 @@
         <v>95</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="58"/>
+    <row r="21" spans="1:5" ht="29.4" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="65"/>
       <c r="B21" s="38"/>
       <c r="C21" s="18" t="s">
         <v>96</v>
@@ -2077,112 +2077,118 @@
         <v>97</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="54" t="s">
+    <row r="22" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="59" t="s">
         <v>98</v>
       </c>
-      <c r="B22" s="54"/>
-      <c r="C22" s="54"/>
-      <c r="D22" s="54"/>
-    </row>
-    <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="59"/>
+      <c r="C22" s="59"/>
+      <c r="D22" s="59"/>
+    </row>
+    <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="9">
         <v>1</v>
       </c>
-      <c r="B23" s="66" t="s">
+      <c r="B23" s="72" t="s">
         <v>39</v>
       </c>
-      <c r="C23" s="67"/>
+      <c r="C23" s="73"/>
       <c r="D23" s="5" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="11">
         <v>2</v>
       </c>
-      <c r="B24" s="50" t="s">
+      <c r="B24" s="55" t="s">
         <v>41</v>
       </c>
-      <c r="C24" s="51"/>
+      <c r="C24" s="56"/>
       <c r="D24" s="7" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="11">
         <v>3</v>
       </c>
-      <c r="B25" s="50" t="s">
+      <c r="B25" s="55" t="s">
         <v>43</v>
       </c>
-      <c r="C25" s="51"/>
+      <c r="C25" s="56"/>
       <c r="D25" s="7" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="11">
         <v>4</v>
       </c>
-      <c r="B26" s="50" t="s">
+      <c r="B26" s="55" t="s">
         <v>45</v>
       </c>
-      <c r="C26" s="51"/>
+      <c r="C26" s="56"/>
       <c r="D26" s="7" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="11">
         <v>5</v>
       </c>
-      <c r="B27" s="50" t="s">
+      <c r="B27" s="55" t="s">
         <v>47</v>
       </c>
-      <c r="C27" s="51"/>
+      <c r="C27" s="56"/>
       <c r="D27" s="7" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="11">
         <v>6</v>
       </c>
-      <c r="B28" s="50" t="s">
+      <c r="B28" s="55" t="s">
         <v>51</v>
       </c>
-      <c r="C28" s="51"/>
+      <c r="C28" s="56"/>
       <c r="D28" s="7" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A29" s="11">
         <v>7</v>
       </c>
-      <c r="B29" s="50" t="s">
+      <c r="B29" s="55" t="s">
         <v>53</v>
       </c>
-      <c r="C29" s="51"/>
+      <c r="C29" s="56"/>
       <c r="D29" s="7" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A30" s="12">
         <v>8</v>
       </c>
-      <c r="B30" s="52" t="s">
+      <c r="B30" s="57" t="s">
         <v>55</v>
       </c>
-      <c r="C30" s="53"/>
+      <c r="C30" s="58"/>
       <c r="D30" s="8" t="s">
         <v>99</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A13:A21"/>
+    <mergeCell ref="A22:D22"/>
+    <mergeCell ref="B23:C23"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A4:A10"/>
     <mergeCell ref="B30:C30"/>
     <mergeCell ref="B24:C24"/>
     <mergeCell ref="B25:C25"/>
@@ -2190,12 +2196,6 @@
     <mergeCell ref="B27:C27"/>
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="B29:C29"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A13:A21"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="B23:C23"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A4:A10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -2205,12 +2205,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1F854E2D-0B73-46F0-A47C-EC8E21F4946D}">
   <dimension ref="A1:C16"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="13.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>105</v>
       </c>
@@ -2221,7 +2221,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -2232,7 +2232,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -2240,7 +2240,7 @@
         <v>46128</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -2248,7 +2248,7 @@
         <v>46135</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" s="46">
         <v>4</v>
       </c>
@@ -2259,7 +2259,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -2267,7 +2267,7 @@
         <v>46149</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -2275,7 +2275,7 @@
         <v>46156</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A8" s="44">
         <v>7</v>
       </c>
@@ -2286,7 +2286,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -2294,7 +2294,7 @@
         <v>46170</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -2302,7 +2302,7 @@
         <v>46177</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A11" s="46">
         <v>10</v>
       </c>
@@ -2313,7 +2313,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -2321,7 +2321,7 @@
         <v>46191</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A13" s="44">
         <v>12</v>
       </c>
@@ -2332,7 +2332,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A14" s="46">
         <v>13</v>
       </c>
@@ -2343,7 +2343,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A15" s="42">
         <v>14</v>
       </c>
@@ -2354,7 +2354,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" s="44">
         <v>15</v>
       </c>

</xml_diff>